<commit_message>
Sync full REST and MQTT documentation updates
</commit_message>
<xml_diff>
--- a/project_resources/analysis_reports/rest_vs_mqtt_field_report.xlsx
+++ b/project_resources/analysis_reports/rest_vs_mqtt_field_report.xlsx
@@ -36,7 +36,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -58,6 +58,11 @@
         <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -71,12 +76,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -442,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -460,7 +466,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>REST operations in openAPISpec2</t>
+          <t>REST operations in RestDeveloperfile</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -484,7 +490,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5">
@@ -504,7 +510,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7">
@@ -524,7 +530,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>760</v>
+        <v>755</v>
       </c>
     </row>
     <row r="9">
@@ -544,7 +550,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11">
@@ -584,7 +590,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>576</v>
+        <v>571</v>
       </c>
     </row>
     <row r="15">
@@ -614,7 +620,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="18">
@@ -637,6 +643,16 @@
         <is>
           <t>Count</t>
         </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Description mismatch</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -650,18 +666,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="7" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="6" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="80" customWidth="1" min="8" max="8"/>
+    <col width="80" customWidth="1" min="9" max="9"/>
     <col width="8" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
@@ -716,6 +732,246 @@
           <t>Detail</t>
         </is>
       </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Description mismatch</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>PUT /cloud/apps/{appname}/autostart</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>setAutostartuserapp</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>autostart_user_app</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>request</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>appname</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Required for MQTT API. Not needed for local REST (use path parameter instead).</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Application name. For REST, the application is identified by the appname path parameter; for MQTT, the application is identified by the appname payload field.</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Description mismatch</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>PUT /cloud/apps/{appname}/pass-through</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>setReqtouserapp</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>set_req_usr_app</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>request</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>userapp</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Name of the target user application.</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>User application name. For REST, the application is identified by the appname path parameter; for MQTT, the application is identified by the userapp payload field.</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Description mismatch</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>PUT /cloud/apps/{appname}/start</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>setStartuserapp</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>start_user_app</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>request</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>appname</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Required for MQTT API. Not needed for local REST (use path parameter instead).</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Application name. For REST, the application is identified by the appname path parameter; for MQTT, the application is identified by the appname payload field.</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Description mismatch</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>PUT /cloud/apps/{appname}/stop</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>setStopuserapp</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>stop_user_app</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>request</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>appname</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Required for MQTT API. Not needed for local REST (use path parameter instead).</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Application name. For REST, the application is identified by the appname path parameter; for MQTT, the application is identified by the appname payload field.</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Description mismatch</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>PUT /cloud/apps/{appname}/uninstall</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>setUninstalluserapp</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>uninstall-user-app</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>request</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>appname</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Required for MQTT API. Not needed for local REST (use path parameter instead).</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Application name. For REST, the application is identified by the appname path parameter; for MQTT, the application is identified by the appname payload field.</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2483,19 +2739,19 @@
         <v>2</v>
       </c>
       <c r="E38" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F38" t="n">
         <v>0</v>
       </c>
       <c r="G38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H38" t="n">
         <v>0</v>
       </c>
       <c r="I38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J38" t="n">
         <v>0</v>
@@ -2505,7 +2761,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>ALIGNED</t>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
@@ -2529,19 +2785,19 @@
         <v>3</v>
       </c>
       <c r="E39" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F39" t="n">
         <v>0</v>
       </c>
       <c r="G39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H39" t="n">
         <v>0</v>
       </c>
       <c r="I39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J39" t="n">
         <v>0</v>
@@ -2551,7 +2807,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>ALIGNED</t>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
@@ -2575,19 +2831,19 @@
         <v>1</v>
       </c>
       <c r="E40" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F40" t="n">
         <v>0</v>
       </c>
       <c r="G40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H40" t="n">
         <v>0</v>
       </c>
       <c r="I40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J40" t="n">
         <v>0</v>
@@ -2597,7 +2853,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>ALIGNED</t>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
@@ -2621,19 +2877,19 @@
         <v>1</v>
       </c>
       <c r="E41" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F41" t="n">
         <v>0</v>
       </c>
       <c r="G41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H41" t="n">
         <v>0</v>
       </c>
       <c r="I41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J41" t="n">
         <v>0</v>
@@ -2643,7 +2899,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>ALIGNED</t>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
@@ -2667,19 +2923,19 @@
         <v>1</v>
       </c>
       <c r="E42" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F42" t="n">
         <v>0</v>
       </c>
       <c r="G42" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H42" t="n">
         <v>0</v>
       </c>
       <c r="I42" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J42" t="n">
         <v>0</v>
@@ -2689,7 +2945,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>ALIGNED</t>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
@@ -42641,17 +42897,17 @@
       </c>
       <c r="M447" t="inlineStr">
         <is>
+          <t>Required for MQTT API. Not needed for local REST (use path parameter instead).</t>
+        </is>
+      </c>
+      <c r="N447" t="inlineStr">
+        <is>
           <t>Application name. For REST, the application is identified by the appname path parameter; for MQTT, the application is identified by the appname payload field.</t>
         </is>
       </c>
-      <c r="N447" t="inlineStr">
-        <is>
-          <t>Application name. For REST, the application is identified by the appname path parameter; for MQTT, the application is identified by the appname payload field.</t>
-        </is>
-      </c>
       <c r="O447" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="P447" t="inlineStr">
@@ -42669,9 +42925,9 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="S447" s="4" t="inlineStr">
-        <is>
-          <t>OK</t>
+      <c r="S447" s="5" t="inlineStr">
+        <is>
+          <t>Description mismatch</t>
         </is>
       </c>
     </row>
@@ -42997,17 +43253,17 @@
       </c>
       <c r="M451" t="inlineStr">
         <is>
+          <t>Name of the target user application.</t>
+        </is>
+      </c>
+      <c r="N451" t="inlineStr">
+        <is>
           <t>User application name. For REST, the application is identified by the appname path parameter; for MQTT, the application is identified by the userapp payload field.</t>
         </is>
       </c>
-      <c r="N451" t="inlineStr">
-        <is>
-          <t>User application name. For REST, the application is identified by the appname path parameter; for MQTT, the application is identified by the userapp payload field.</t>
-        </is>
-      </c>
       <c r="O451" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="P451" t="inlineStr">
@@ -43025,9 +43281,9 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="S451" s="4" t="inlineStr">
-        <is>
-          <t>OK</t>
+      <c r="S451" s="5" t="inlineStr">
+        <is>
+          <t>Description mismatch</t>
         </is>
       </c>
     </row>
@@ -43086,17 +43342,17 @@
       </c>
       <c r="M452" t="inlineStr">
         <is>
+          <t>Required for MQTT API. Not needed for local REST (use path parameter instead).</t>
+        </is>
+      </c>
+      <c r="N452" t="inlineStr">
+        <is>
           <t>Application name. For REST, the application is identified by the appname path parameter; for MQTT, the application is identified by the appname payload field.</t>
         </is>
       </c>
-      <c r="N452" t="inlineStr">
-        <is>
-          <t>Application name. For REST, the application is identified by the appname path parameter; for MQTT, the application is identified by the appname payload field.</t>
-        </is>
-      </c>
       <c r="O452" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="P452" t="inlineStr">
@@ -43114,9 +43370,9 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="S452" s="4" t="inlineStr">
-        <is>
-          <t>OK</t>
+      <c r="S452" s="5" t="inlineStr">
+        <is>
+          <t>Description mismatch</t>
         </is>
       </c>
     </row>
@@ -43175,17 +43431,17 @@
       </c>
       <c r="M453" t="inlineStr">
         <is>
+          <t>Required for MQTT API. Not needed for local REST (use path parameter instead).</t>
+        </is>
+      </c>
+      <c r="N453" t="inlineStr">
+        <is>
           <t>Application name. For REST, the application is identified by the appname path parameter; for MQTT, the application is identified by the appname payload field.</t>
         </is>
       </c>
-      <c r="N453" t="inlineStr">
-        <is>
-          <t>Application name. For REST, the application is identified by the appname path parameter; for MQTT, the application is identified by the appname payload field.</t>
-        </is>
-      </c>
       <c r="O453" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="P453" t="inlineStr">
@@ -43203,9 +43459,9 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="S453" s="4" t="inlineStr">
-        <is>
-          <t>OK</t>
+      <c r="S453" s="5" t="inlineStr">
+        <is>
+          <t>Description mismatch</t>
         </is>
       </c>
     </row>
@@ -43264,17 +43520,17 @@
       </c>
       <c r="M454" t="inlineStr">
         <is>
+          <t>Required for MQTT API. Not needed for local REST (use path parameter instead).</t>
+        </is>
+      </c>
+      <c r="N454" t="inlineStr">
+        <is>
           <t>Application name. For REST, the application is identified by the appname path parameter; for MQTT, the application is identified by the appname payload field.</t>
         </is>
       </c>
-      <c r="N454" t="inlineStr">
-        <is>
-          <t>Application name. For REST, the application is identified by the appname path parameter; for MQTT, the application is identified by the appname payload field.</t>
-        </is>
-      </c>
       <c r="O454" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="P454" t="inlineStr">
@@ -43292,9 +43548,9 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="S454" s="4" t="inlineStr">
-        <is>
-          <t>OK</t>
+      <c r="S454" s="5" t="inlineStr">
+        <is>
+          <t>Description mismatch</t>
         </is>
       </c>
     </row>
@@ -70724,17 +70980,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="6" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
     <col width="5" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -70776,6 +71032,166 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Top issues</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>PUT /cloud/apps/{appname}/autostart</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>autostart_user_app</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Description mismatch</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>PUT /cloud/apps/{appname}/pass-through</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>set_req_usr_app</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Description mismatch</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>PUT /cloud/apps/{appname}/start</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>start_user_app</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Description mismatch</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>PUT /cloud/apps/{appname}/stop</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>stop_user_app</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Description mismatch</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>PUT /cloud/apps/{appname}/uninstall</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>uninstall-user-app</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Description mismatch</t>
         </is>
       </c>
     </row>
@@ -70868,18 +71284,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="7" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="6" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="80" customWidth="1" min="8" max="8"/>
+    <col width="80" customWidth="1" min="9" max="9"/>
     <col width="8" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
@@ -70934,6 +71350,246 @@
           <t>Detail</t>
         </is>
       </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Description mismatch</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>PUT /cloud/apps/{appname}/start</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>setStartuserapp</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>start_user_app</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>request</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>appname</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Required for MQTT API. Not needed for local REST (use path parameter instead).</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Application name. For REST, the application is identified by the appname path parameter; for MQTT, the application is identified by the appname payload field.</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Description mismatch</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>PUT /cloud/apps/{appname}/stop</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>setStopuserapp</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>stop_user_app</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>request</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>appname</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Required for MQTT API. Not needed for local REST (use path parameter instead).</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Application name. For REST, the application is identified by the appname path parameter; for MQTT, the application is identified by the appname payload field.</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Description mismatch</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>PUT /cloud/apps/{appname}/autostart</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>setAutostartuserapp</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>autostart_user_app</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>request</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>appname</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Required for MQTT API. Not needed for local REST (use path parameter instead).</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Application name. For REST, the application is identified by the appname path parameter; for MQTT, the application is identified by the appname payload field.</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Description mismatch</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>PUT /cloud/apps/{appname}/pass-through</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>setReqtouserapp</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>set_req_usr_app</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>request</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>userapp</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Name of the target user application.</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>User application name. For REST, the application is identified by the appname path parameter; for MQTT, the application is identified by the userapp payload field.</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Description mismatch</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>PUT /cloud/apps/{appname}/uninstall</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>setUninstalluserapp</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>uninstall-user-app</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>request</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>appname</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Required for MQTT API. Not needed for local REST (use path parameter instead).</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Application name. For REST, the application is identified by the appname path parameter; for MQTT, the application is identified by the appname payload field.</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>